<commit_message>
synced with main branch
</commit_message>
<xml_diff>
--- a/MMT_Automation/src/test/resources/data/BiswayanNath_AutomationTesting.xlsx
+++ b/MMT_Automation/src/test/resources/data/BiswayanNath_AutomationTesting.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\biswa\Downloads\Capg\Sprint\MMT_Automation\src\test\resources\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A86C802-5559-40F9-89E7-3FD89BC2E953}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69C2A92C-A7A5-448A-99EC-1D8AE80FCC41}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{CF9C7236-DFC9-4ECB-B16E-6D2432981843}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -108,9 +108,6 @@
 4. 2 Adults, 1 Room</t>
   </si>
   <si>
-    <t>It should not accept the specified details.</t>
-  </si>
-  <si>
     <t>TC_MakeMyTrip_03</t>
   </si>
   <si>
@@ -260,6 +257,9 @@
     <t>1. Click on Disney Cruise.
 2. Click on View All.
 3. Click on the first package from Disney Cruise.</t>
+  </si>
+  <si>
+    <t>It should not accept the invalid details.</t>
   </si>
 </sst>
 </file>
@@ -1133,13 +1133,13 @@
         <v>14</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D2" s="7" t="s">
         <v>15</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F2" s="8" t="s">
         <v>16</v>
@@ -1157,7 +1157,7 @@
       <c r="K2" s="9"/>
       <c r="L2" s="10"/>
       <c r="M2" s="12" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="135">
@@ -1168,7 +1168,7 @@
         <v>14</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>21</v>
@@ -1180,10 +1180,10 @@
         <v>23</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>24</v>
+        <v>69</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I3" s="9" t="s">
         <v>19</v>
@@ -1192,72 +1192,72 @@
       <c r="K3" s="9"/>
       <c r="L3" s="10"/>
       <c r="M3" s="12" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="150">
       <c r="A4" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>14</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D4" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="F4" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="G4" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="H4" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="I4" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="9" t="s">
-        <v>31</v>
-      </c>
       <c r="J4" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="K4" s="9" t="s">
         <v>30</v>
-      </c>
-      <c r="K4" s="9" t="s">
-        <v>31</v>
       </c>
       <c r="L4" s="10"/>
       <c r="M4" s="12" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="60">
       <c r="A5" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="C5" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="D5" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C5" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="D5" s="7" t="s">
+      <c r="E5" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="F5" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="G5" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="H5" s="7" t="s">
         <v>37</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>38</v>
       </c>
       <c r="I5" s="9" t="s">
         <v>19</v>
@@ -1266,33 +1266,33 @@
       <c r="K5" s="9"/>
       <c r="L5" s="10"/>
       <c r="M5" s="12" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="105">
       <c r="A6" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="D6" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="B6" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="D6" s="7" t="s">
+      <c r="E6" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="G6" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="E6" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="G6" s="7" t="s">
+      <c r="H6" s="7" t="s">
         <v>41</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>42</v>
       </c>
       <c r="I6" s="9" t="s">
         <v>19</v>
@@ -1301,33 +1301,33 @@
       <c r="K6" s="9"/>
       <c r="L6" s="10"/>
       <c r="M6" s="12" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="105">
       <c r="A7" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="D7" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B7" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="D7" s="7" t="s">
+      <c r="E7" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="G7" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="E7" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="G7" s="7" t="s">
+      <c r="H7" s="7" t="s">
         <v>45</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>46</v>
       </c>
       <c r="I7" s="9" t="s">
         <v>19</v>
@@ -1336,33 +1336,33 @@
       <c r="K7" s="9"/>
       <c r="L7" s="10"/>
       <c r="M7" s="12" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="60">
       <c r="A8" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="C8" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="D8" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="C8" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="D8" s="7" t="s">
+      <c r="E8" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="F8" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="G8" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="F8" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="G8" s="7" t="s">
+      <c r="H8" s="7" t="s">
         <v>51</v>
-      </c>
-      <c r="H8" s="7" t="s">
-        <v>52</v>
       </c>
       <c r="I8" s="9" t="s">
         <v>19</v>
@@ -1371,33 +1371,33 @@
       <c r="K8" s="9"/>
       <c r="L8" s="10"/>
       <c r="M8" s="12" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="60">
       <c r="A9" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="D9" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="B9" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="D9" s="7" t="s">
+      <c r="E9" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="F9" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="G9" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="F9" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="G9" s="7" t="s">
+      <c r="H9" s="7" t="s">
         <v>56</v>
-      </c>
-      <c r="H9" s="7" t="s">
-        <v>57</v>
       </c>
       <c r="I9" s="9" t="s">
         <v>19</v>
@@ -1406,33 +1406,33 @@
       <c r="K9" s="9"/>
       <c r="L9" s="10"/>
       <c r="M9" s="12" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="120">
       <c r="A10" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="D10" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B10" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="D10" s="7" t="s">
+      <c r="E10" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="G10" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="E10" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="F10" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="G10" s="7" t="s">
+      <c r="H10" s="7" t="s">
         <v>60</v>
-      </c>
-      <c r="H10" s="7" t="s">
-        <v>61</v>
       </c>
       <c r="I10" s="9" t="s">
         <v>19</v>
@@ -1441,7 +1441,7 @@
       <c r="K10" s="9"/>
       <c r="L10" s="10"/>
       <c r="M10" s="12" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>